<commit_message>
actualiza acumulados 22/06/2026 11:47
</commit_message>
<xml_diff>
--- a/Pruebas calificadas/COLEGIO FRANCISCO DE MIRANDA-703_CALIFICADO.xlsx
+++ b/Pruebas calificadas/COLEGIO FRANCISCO DE MIRANDA-703_CALIFICADO.xlsx
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AZ63"/>
+  <dimension ref="A1:AZ65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -15716,6 +15716,352 @@
         <v/>
       </c>
     </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>111001014974</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>COLEGIO FRANCISCO DE MIRANDA (IED)</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>DANIEL FELIPE PEREZ PARRADO</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>1012922767</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>703</v>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>LENGUAJE</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr"/>
+      <c r="P64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Q64" s="2" t="inlineStr"/>
+      <c r="R64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="S64" s="2" t="inlineStr"/>
+      <c r="T64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="U64" s="2" t="inlineStr"/>
+      <c r="V64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="W64" s="2" t="inlineStr"/>
+      <c r="X64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Y64" s="2" t="inlineStr"/>
+      <c r="Z64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AA64" s="2" t="inlineStr"/>
+      <c r="AB64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AC64" s="2" t="inlineStr"/>
+      <c r="AD64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AE64" s="2" t="inlineStr"/>
+      <c r="AF64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AG64" s="2" t="inlineStr"/>
+      <c r="AH64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AI64" s="2" t="inlineStr"/>
+      <c r="AJ64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AK64" s="2" t="inlineStr"/>
+      <c r="AL64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AM64" s="2" t="inlineStr"/>
+      <c r="AN64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AO64" s="2" t="inlineStr"/>
+      <c r="AP64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AQ64" s="2" t="inlineStr"/>
+      <c r="AR64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AS64" s="2" t="inlineStr"/>
+      <c r="AT64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AU64" s="2" t="inlineStr"/>
+      <c r="AV64" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AW64" s="5">
+        <f>COUNTIF(J64:AV64,"CORRECTO")</f>
+        <v/>
+      </c>
+      <c r="AX64" s="5">
+        <f>COUNTIF(J64:AV64,"INCORRECTO")</f>
+        <v/>
+      </c>
+      <c r="AY64" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="AZ64" s="6">
+        <f>AW64/AY64</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>111001014974</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>COLEGIO FRANCISCO DE MIRANDA (IED)</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>JUAN ESTEBAN VALLEJO ROMERO</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>1146129401</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>703</v>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>LENGUAJE</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr"/>
+      <c r="P65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="inlineStr"/>
+      <c r="R65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="S65" s="2" t="inlineStr"/>
+      <c r="T65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="U65" s="2" t="inlineStr"/>
+      <c r="V65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="W65" s="2" t="inlineStr"/>
+      <c r="X65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="Y65" s="2" t="inlineStr"/>
+      <c r="Z65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AA65" s="2" t="inlineStr"/>
+      <c r="AB65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AC65" s="2" t="inlineStr"/>
+      <c r="AD65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AE65" s="2" t="inlineStr"/>
+      <c r="AF65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AG65" s="2" t="inlineStr"/>
+      <c r="AH65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AI65" s="2" t="inlineStr"/>
+      <c r="AJ65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AK65" s="2" t="inlineStr"/>
+      <c r="AL65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AM65" s="2" t="inlineStr"/>
+      <c r="AN65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AO65" s="2" t="inlineStr"/>
+      <c r="AP65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AQ65" s="2" t="inlineStr"/>
+      <c r="AR65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AS65" s="2" t="inlineStr"/>
+      <c r="AT65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AU65" s="2" t="inlineStr"/>
+      <c r="AV65" s="4" t="inlineStr">
+        <is>
+          <t>INCORRECTO</t>
+        </is>
+      </c>
+      <c r="AW65" s="5">
+        <f>COUNTIF(J65:AV65,"CORRECTO")</f>
+        <v/>
+      </c>
+      <c r="AX65" s="5">
+        <f>COUNTIF(J65:AV65,"INCORRECTO")</f>
+        <v/>
+      </c>
+      <c r="AY65" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="AZ65" s="6">
+        <f>AW65/AY65</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>